<commit_message>
add example wf and run descriptions
</commit_message>
<xml_diff>
--- a/workflows/fairagroUC6/isa.workflow.xlsx
+++ b/workflows/fairagroUC6/isa.workflow.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
   <si>
     <t>WORKFLOW</t>
   </si>
@@ -28,42 +28,83 @@
     <t>Workflow Description</t>
   </si>
   <si>
+    <t xml:space="preserve">## Introduction
+The repository contains computational workflows for crop simulation modelling created using the [FAIRagro Scientific Workflow Infrastructure (SciWIn)](https://github.com/fairagro/sciwin) tool.
+Workflows are expressed in [CWL v1.2](https://www.commonwl.org/) and executed with [s4n](https://github.com/fairagro/sciwin), which runs each tool step inside a Docker container.
+### Implemented Workflow
+The full pipeline takes field observations (UAV-derived NDVI, crop calendar, and field metadata) and produces ready-to-run DSSAT crop simulation files alongside a results plot:
+![CSM Workflow diagram](documentation/csm_workflow.png)</t>
+  </si>
+  <si>
     <t>Workflow Type</t>
   </si>
   <si>
+    <t>CWL</t>
+  </si>
+  <si>
     <t>Workflow Type Term Accession Number</t>
   </si>
   <si>
+    <t>http://purl.obolibrary.org/obo/EDAM_3857</t>
+  </si>
+  <si>
     <t>Workflow Type Term Source REF</t>
   </si>
   <si>
+    <t>edam</t>
+  </si>
+  <si>
     <t>Workflow Sub Workflow Identifiers</t>
   </si>
   <si>
     <t>Workflow URI</t>
   </si>
   <si>
+    <t>https://raw.githubusercontent.com/Brilator/fairagroUC6-workflows-ARC/refs/heads/main/workflows/fairagroUC6/workflow.cwl</t>
+  </si>
+  <si>
     <t>Workflow Version</t>
   </si>
   <si>
+    <t>0.1.0</t>
+  </si>
+  <si>
     <t>Workflow Parameters Name</t>
   </si>
   <si>
+    <t>Crop;crop modelling;simulation models</t>
+  </si>
+  <si>
     <t>Workflow Parameters Term Accession Number</t>
   </si>
   <si>
+    <t>NCIT:C111162;C:9000024;C:24242</t>
+  </si>
+  <si>
     <t>Workflow Parameters Term Source REF</t>
   </si>
   <si>
+    <t>NCIT;C;C</t>
+  </si>
+  <si>
     <t>Workflow Components Name</t>
   </si>
   <si>
+    <t>Docker image (EDAM:3973);DSSAT</t>
+  </si>
+  <si>
     <t>Workflow Components Type</t>
   </si>
   <si>
+    <t>;Simulation Files</t>
+  </si>
+  <si>
     <t>Workflow Components Type Term Accession Number</t>
   </si>
   <si>
+    <t>;</t>
+  </si>
+  <si>
     <t>Workflow Components Type Term Source REF</t>
   </si>
   <si>
@@ -73,15 +114,27 @@
     <t>workflows/fairagroUC6/isa.workflow.xlsx</t>
   </si>
   <si>
+    <t>Comment[Critic]</t>
+  </si>
+  <si>
+    <t>Don't use comments. They are bad style.</t>
+  </si>
+  <si>
     <t>WORKFLOW CONTACTS</t>
   </si>
   <si>
     <t>Workflow Person Last Name</t>
   </si>
   <si>
+    <t>Mureithi</t>
+  </si>
+  <si>
     <t>Workflow Person First Name</t>
   </si>
   <si>
+    <t>Joseph</t>
+  </si>
+  <si>
     <t>Workflow Person Mid Initials</t>
   </si>
   <si>
@@ -98,6 +151,9 @@
   </si>
   <si>
     <t>Workflow Person Affiliation</t>
+  </si>
+  <si>
+    <t>Technical University of Munich</t>
   </si>
   <si>
     <t>Workflow Person Roles</t>
@@ -458,7 +514,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -474,147 +530,206 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="B13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="B14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="B15" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>29</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>32</v>
+      </c>
+      <c r="B19" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+      <c r="B21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>37</v>
+      </c>
+      <c r="B22" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>29</v>
+        <v>44</v>
+      </c>
+      <c r="B28" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>